<commit_message>
Add example data rows to all xlsx templates
- Jadwal Imam: 7 example rows (daily schedule + Jumat special)
- Kas: 6 example transactions + 1 monthly recap
- Inventaris: 10 example items + 3 change log entries
- Example rows highlighted light green, headers gray
- 10 empty rows for user data after examples
</commit_message>
<xml_diff>
--- a/docs/public/template/inventaris-barang.xlsx
+++ b/docs/public/template/inventaris-barang.xlsx
@@ -405,11 +405,11 @@
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
     <col min="11" max="11" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -436,7 +436,7 @@
         <v>Kondisi</v>
       </c>
       <c r="H1" t="str">
-        <v>Tanggal Perolehan</v>
+        <v>Tgl Perolehan</v>
       </c>
       <c r="I1" t="str">
         <v>Sumber</v>
@@ -450,69 +450,69 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Karpet sajadah (1,5m x 3m)</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Perlengkapan Shalat</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>4</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>Lembar</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>Ruang utama — depan</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>15/03/2024</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>Sumbangan</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>✓</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>Sumbangan Bpk. Haji Rahman</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>Al-Quran (cetakan Madinah)</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Perlengkapan Shalat</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>Rak Al-Quran</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>01/01/2023</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>✓</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -520,136 +520,136 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Mukena (dewasa)</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Perlengkapan Shalat</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>Lemari belakang</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>Cukup</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>01/01/2023</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J4" t="str">
         <v/>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>2 agak luntur, perlu diganti tahun depan</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>Kipas Angin Maspion 16"</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Listrik &amp; Air</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>Ruang utama (2), Wudu (1)</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>10/06/2024</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>✓</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>Kipas wudu diperbaiki Mei 2025</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>Pengeras Suara TOA 30W</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>Audio</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>Set</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>Atas mimbar</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>01/01/2023</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>Sumbangan</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>✓</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>Termasuk mic + kabel</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>Sapu lidi</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Kebersihan</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>Belakang pintu</v>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>Tidak Diketahui</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>Tidak Diketahui</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -660,142 +660,142 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>Ember + Pel</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Kebersihan</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>Set</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>Ruang wudu</v>
       </c>
       <c r="G8" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>05/05/2025</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J8" t="str">
         <v/>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>Baru dibeli</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v/>
+        <v>Rak Sepatu (kayu, 4 tingkat)</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>Perabot</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>Depan pintu masuk</v>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>Cukup</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>01/01/2023</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>✓</v>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>Agak goyang, perlu diperkuat</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>Kotak Infak (kayu, berkunci)</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>Dokumen</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>Dekat pintu + pojok</v>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>01/01/2023</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>✓</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>Kunci dipegang bendahara</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>Buku Kas</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>Dokumen</v>
       </c>
       <c r="D11" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>Buah</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>Lemari bendahara</v>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>Baik</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>01/01/2025</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>Beli</v>
       </c>
       <c r="J11" t="str">
         <v/>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>Periode 2025, diganti setiap tahun</v>
       </c>
     </row>
     <row r="12">
@@ -1157,12 +1157,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1177,7 +1177,7 @@
         <v>Jenis Perubahan</v>
       </c>
       <c r="D1" t="str">
-        <v>Keterangan Perubahan</v>
+        <v>Keterangan</v>
       </c>
       <c r="E1" t="str">
         <v>Ditangani Oleh</v>
@@ -1185,53 +1185,53 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>10/05/2025</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Kipas Angin Maspion (wudu)</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Diperbaiki</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>Kipas di ruang wudu macet. Ganti dinamo. Biaya Rp 200.000 dari kas.</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>Bpk. Hasan</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>05/06/2025</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>Karpet sajadah (2 lembar)</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Rusak</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>Karpet robek di bagian tengah. Tidak bisa diperbaiki — diganti baru.</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>Bpk. Hasan</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v/>
+        <v>20/06/2025</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Karpet sajadah (baru, 4 lembar)</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Ditambah</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>Beli 4 lembar karpet baru. Pengganti yang robek + tambahan. Biaya Rp 800.000.</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>Bpk. Hasan</v>
       </c>
     </row>
     <row r="5">
@@ -1404,128 +1404,9 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v/>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v/>
-      </c>
-      <c r="B16" t="str">
-        <v/>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v/>
-      </c>
-      <c r="B17" t="str">
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <v/>
-      </c>
-      <c r="E18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v/>
-      </c>
-      <c r="B19" t="str">
-        <v/>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <v/>
-      </c>
-      <c r="E19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v/>
-      </c>
-      <c r="B20" t="str">
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v/>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Embed Excel formulas for dynamic calculation
Kas template:
- Saldo column: running balance formula (=IF + previous row)
- Rekap Bulanan: SUMIF cross-sheet references to Buku Kas Harian
- Saldo Akhir: D+B-C formula

Open in Excel/WPS/Sheets — formulas calculate automatically
</commit_message>
<xml_diff>
--- a/docs/public/template/inventaris-barang.xlsx
+++ b/docs/public/template/inventaris-barang.xlsx
@@ -401,16 +401,16 @@
   <dimension ref="A1:K21"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" customWidth="1"/>
-    <col min="11" max="11" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="6.83203125" customWidth="1"/>
+    <col min="11" max="11" width="32.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,7 +449,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="str">
@@ -458,7 +458,7 @@
       <c r="C2" t="str">
         <v>Perlengkapan Shalat</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2">
         <v>4</v>
       </c>
       <c r="E2" t="str">
@@ -480,11 +480,11 @@
         <v>✓</v>
       </c>
       <c r="K2" t="str">
-        <v>Sumbangan Bpk. Haji Rahman</v>
+        <v>Bpk. Haji Rahman</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="str">
@@ -493,7 +493,7 @@
       <c r="C3" t="str">
         <v>Perlengkapan Shalat</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3">
         <v>10</v>
       </c>
       <c r="E3" t="str">
@@ -519,7 +519,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="str">
@@ -528,7 +528,7 @@
       <c r="C4" t="str">
         <v>Perlengkapan Shalat</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4">
         <v>5</v>
       </c>
       <c r="E4" t="str">
@@ -550,11 +550,11 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v>2 agak luntur, perlu diganti tahun depan</v>
+        <v>2 luntur, ganti 2026</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="str">
@@ -563,7 +563,7 @@
       <c r="C5" t="str">
         <v>Listrik &amp; Air</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5">
         <v>3</v>
       </c>
       <c r="E5" t="str">
@@ -585,11 +585,11 @@
         <v>✓</v>
       </c>
       <c r="K5" t="str">
-        <v>Kipas wudu diperbaiki Mei 2025</v>
+        <v>Kipas wudu ganti dinamo Mei 2025</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="str">
@@ -598,7 +598,7 @@
       <c r="C6" t="str">
         <v>Audio</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="str">
@@ -624,7 +624,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="str">
@@ -633,7 +633,7 @@
       <c r="C7" t="str">
         <v>Kebersihan</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="str">
@@ -646,10 +646,10 @@
         <v>Baik</v>
       </c>
       <c r="H7" t="str">
-        <v>Tidak Diketahui</v>
+        <v/>
       </c>
       <c r="I7" t="str">
-        <v>Tidak Diketahui</v>
+        <v/>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -659,7 +659,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="str">
@@ -668,7 +668,7 @@
       <c r="C8" t="str">
         <v>Kebersihan</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D8">
         <v>2</v>
       </c>
       <c r="E8" t="str">
@@ -690,11 +690,11 @@
         <v/>
       </c>
       <c r="K8" t="str">
-        <v>Baru dibeli</v>
+        <v>Baru</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="str">
@@ -703,14 +703,14 @@
       <c r="C9" t="str">
         <v>Perabot</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="str">
         <v>Buah</v>
       </c>
       <c r="F9" t="str">
-        <v>Depan pintu masuk</v>
+        <v>Depan pintu</v>
       </c>
       <c r="G9" t="str">
         <v>Cukup</v>
@@ -725,11 +725,11 @@
         <v>✓</v>
       </c>
       <c r="K9" t="str">
-        <v>Agak goyang, perlu diperkuat</v>
+        <v>Agak goyang</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
+      <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="str">
@@ -738,7 +738,7 @@
       <c r="C10" t="str">
         <v>Dokumen</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D10">
         <v>2</v>
       </c>
       <c r="E10" t="str">
@@ -760,11 +760,11 @@
         <v>✓</v>
       </c>
       <c r="K10" t="str">
-        <v>Kunci dipegang bendahara</v>
+        <v>Kunci di bendahara</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
+      <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="str">
@@ -773,7 +773,7 @@
       <c r="C11" t="str">
         <v>Dokumen</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D11">
         <v>1</v>
       </c>
       <c r="E11" t="str">
@@ -795,357 +795,7 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v>Periode 2025, diganti setiap tahun</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <v/>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
-      <c r="J12" t="str">
-        <v/>
-      </c>
-      <c r="K12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v/>
-      </c>
-      <c r="B13" t="str">
-        <v/>
-      </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
-      <c r="K13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v/>
-      </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
-      <c r="H14" t="str">
-        <v/>
-      </c>
-      <c r="I14" t="str">
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
-      <c r="K14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v/>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
-      <c r="E15" t="str">
-        <v/>
-      </c>
-      <c r="F15" t="str">
-        <v/>
-      </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
-      <c r="K15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v/>
-      </c>
-      <c r="B16" t="str">
-        <v/>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
-        <v/>
-      </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-      <c r="H16" t="str">
-        <v/>
-      </c>
-      <c r="I16" t="str">
-        <v/>
-      </c>
-      <c r="J16" t="str">
-        <v/>
-      </c>
-      <c r="K16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v/>
-      </c>
-      <c r="B17" t="str">
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
-        <v/>
-      </c>
-      <c r="G17" t="str">
-        <v/>
-      </c>
-      <c r="H17" t="str">
-        <v/>
-      </c>
-      <c r="I17" t="str">
-        <v/>
-      </c>
-      <c r="J17" t="str">
-        <v/>
-      </c>
-      <c r="K17" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <v/>
-      </c>
-      <c r="E18" t="str">
-        <v/>
-      </c>
-      <c r="F18" t="str">
-        <v/>
-      </c>
-      <c r="G18" t="str">
-        <v/>
-      </c>
-      <c r="H18" t="str">
-        <v/>
-      </c>
-      <c r="I18" t="str">
-        <v/>
-      </c>
-      <c r="J18" t="str">
-        <v/>
-      </c>
-      <c r="K18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v/>
-      </c>
-      <c r="B19" t="str">
-        <v/>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <v/>
-      </c>
-      <c r="E19" t="str">
-        <v/>
-      </c>
-      <c r="F19" t="str">
-        <v/>
-      </c>
-      <c r="G19" t="str">
-        <v/>
-      </c>
-      <c r="H19" t="str">
-        <v/>
-      </c>
-      <c r="I19" t="str">
-        <v/>
-      </c>
-      <c r="J19" t="str">
-        <v/>
-      </c>
-      <c r="K19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v/>
-      </c>
-      <c r="B20" t="str">
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
-        <v/>
-      </c>
-      <c r="G20" t="str">
-        <v/>
-      </c>
-      <c r="H20" t="str">
-        <v/>
-      </c>
-      <c r="I20" t="str">
-        <v/>
-      </c>
-      <c r="J20" t="str">
-        <v/>
-      </c>
-      <c r="K20" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v/>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
-        <v/>
-      </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
-      <c r="H21" t="str">
-        <v/>
-      </c>
-      <c r="I21" t="str">
-        <v/>
-      </c>
-      <c r="J21" t="str">
-        <v/>
-      </c>
-      <c r="K21" t="str">
-        <v/>
+        <v>Periode 2025</v>
       </c>
     </row>
   </sheetData>
@@ -1160,9 +810,9 @@
   <dimension ref="A1:E14"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1194,7 +844,7 @@
         <v>Diperbaiki</v>
       </c>
       <c r="D2" t="str">
-        <v>Kipas di ruang wudu macet. Ganti dinamo. Biaya Rp 200.000 dari kas.</v>
+        <v>Macet. Ganti dinamo. Biaya Rp 200.000 dari kas.</v>
       </c>
       <c r="E2" t="str">
         <v>Bpk. Hasan</v>
@@ -1211,7 +861,7 @@
         <v>Rusak</v>
       </c>
       <c r="D3" t="str">
-        <v>Karpet robek di bagian tengah. Tidak bisa diperbaiki — diganti baru.</v>
+        <v>Robek tengah. Sudah diganti baru.</v>
       </c>
       <c r="E3" t="str">
         <v>Bpk. Hasan</v>
@@ -1228,180 +878,10 @@
         <v>Ditambah</v>
       </c>
       <c r="D4" t="str">
-        <v>Beli 4 lembar karpet baru. Pengganti yang robek + tambahan. Biaya Rp 800.000.</v>
+        <v>Pengganti + tambahan. Rp 800.000.</v>
       </c>
       <c r="E4" t="str">
         <v>Bpk. Hasan</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v/>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v/>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v/>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-      <c r="B11" t="str">
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <v/>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v/>
-      </c>
-      <c r="B13" t="str">
-        <v/>
-      </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>